<commit_message>
Project 20: generator v2 menanam kelima fakta data rancangan (Cpk<1,33, penurunan PT-02 7 hari, nilai tidak wajar, file kosong, kolom hilang)
Pindai jendela penurunan menggantikan pindai titik ubah; sidik jari diperbarui.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YpKXFN1b3yUWd7Emtd6MU
</commit_message>
<xml_diff>
--- a/project/outputs/reconciliation.xlsx
+++ b/project/outputs/reconciliation.xlsx
@@ -466,13 +466,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3531</v>
+        <v>3401</v>
       </c>
       <c r="E2" t="n">
-        <v>3578</v>
+        <v>3528</v>
       </c>
       <c r="F2" t="n">
-        <v>47</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8474.066468422543</v>
+        <v>8581.919288444575</v>
       </c>
       <c r="E3" t="n">
-        <v>8199.872680128565</v>
+        <v>8305.5497125</v>
       </c>
       <c r="F3" t="n">
-        <v>-274.1937882939783</v>
+        <v>-276.3695759445745</v>
       </c>
     </row>
     <row r="4">
@@ -518,13 +518,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4823.1</v>
+        <v>5702.6</v>
       </c>
       <c r="E4" t="n">
-        <v>6.7691</v>
+        <v>-3058</v>
       </c>
       <c r="F4" t="n">
-        <v>-4816.3309</v>
+        <v>-8760.6</v>
       </c>
     </row>
     <row r="5">
@@ -544,13 +544,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>11642.9</v>
+        <v>11722.8</v>
       </c>
       <c r="E5" t="n">
-        <v>11642.9</v>
+        <v>29472.3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>17749.5</v>
       </c>
     </row>
     <row r="6">
@@ -570,13 +570,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.580154876688126</v>
+        <v>2.734510112171457</v>
       </c>
       <c r="E6" t="n">
-        <v>1.306170942905664</v>
+        <v>0.9022634204720315</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.273983933782461</v>
+        <v>-1.832246691699425</v>
       </c>
     </row>
     <row r="7">
@@ -599,10 +599,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03074343208496367</v>
+        <v>0.05413832199546485</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03074343208496367</v>
+        <v>0.05413832199546485</v>
       </c>
     </row>
     <row r="8">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3854</v>
+        <v>3721</v>
       </c>
       <c r="E8" t="n">
-        <v>3936</v>
+        <v>3892</v>
       </c>
       <c r="F8" t="n">
-        <v>82</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
@@ -648,13 +648,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7067.120160871822</v>
+        <v>7151.974872346143</v>
       </c>
       <c r="E9" t="n">
-        <v>6906.363159400407</v>
+        <v>7057.344121402878</v>
       </c>
       <c r="F9" t="n">
-        <v>-160.7570014714147</v>
+        <v>-94.63075094326541</v>
       </c>
     </row>
     <row r="10">
@@ -674,13 +674,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4068.8</v>
+        <v>3818.4</v>
       </c>
       <c r="E10" t="n">
-        <v>5.209</v>
+        <v>-442</v>
       </c>
       <c r="F10" t="n">
-        <v>-4063.591</v>
+        <v>-4260.4</v>
       </c>
     </row>
     <row r="11">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10331.4</v>
+        <v>10086.3</v>
       </c>
       <c r="E11" t="n">
-        <v>10331.4</v>
+        <v>29954.3</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>19868</v>
       </c>
     </row>
     <row r="12">
@@ -726,13 +726,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.058126494737123</v>
+        <v>2.123856983079873</v>
       </c>
       <c r="E12" t="n">
-        <v>1.313026684593014</v>
+        <v>0.7704692736255384</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.7450998101441093</v>
+        <v>-1.353387709454334</v>
       </c>
     </row>
     <row r="13">
@@ -755,10 +755,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.02235772357723577</v>
+        <v>0.0447070914696814</v>
       </c>
       <c r="F13" t="n">
-        <v>0.02235772357723577</v>
+        <v>0.0447070914696814</v>
       </c>
     </row>
     <row r="14">
@@ -778,13 +778,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3584</v>
+        <v>3412</v>
       </c>
       <c r="E14" t="n">
-        <v>3639</v>
+        <v>3577</v>
       </c>
       <c r="F14" t="n">
-        <v>55</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15">
@@ -804,13 +804,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8155.996261160714</v>
+        <v>8300.667233294256</v>
       </c>
       <c r="E15" t="n">
-        <v>7918.904002665568</v>
+        <v>8094.700690159352</v>
       </c>
       <c r="F15" t="n">
-        <v>-237.0922584951459</v>
+        <v>-205.966543134904</v>
       </c>
     </row>
     <row r="16">
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5082.4</v>
+        <v>4811.1</v>
       </c>
       <c r="E16" t="n">
-        <v>6.1847</v>
+        <v>-481.1</v>
       </c>
       <c r="F16" t="n">
-        <v>-5076.2153</v>
+        <v>-5292.200000000001</v>
       </c>
     </row>
     <row r="17">
@@ -859,10 +859,10 @@
         <v>11388.2</v>
       </c>
       <c r="E17" t="n">
-        <v>11388.2</v>
+        <v>29515.3</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>18127.1</v>
       </c>
     </row>
     <row r="18">
@@ -882,13 +882,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.447423769172285</v>
+        <v>2.564694707772915</v>
       </c>
       <c r="E18" t="n">
-        <v>1.298387306189422</v>
+        <v>0.8038623471140007</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.149036462982862</v>
+        <v>-1.760832360658914</v>
       </c>
     </row>
     <row r="19">
@@ -911,10 +911,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0.02967848309975268</v>
+        <v>0.06094492591557171</v>
       </c>
       <c r="F19" t="n">
-        <v>0.02967848309975268</v>
+        <v>0.06094492591557171</v>
       </c>
     </row>
     <row r="20">
@@ -934,13 +934,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3507</v>
+        <v>3366</v>
       </c>
       <c r="E20" t="n">
-        <v>3516</v>
+        <v>3444</v>
       </c>
       <c r="F20" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21">
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6676.220387795836</v>
+        <v>6758.616904337493</v>
       </c>
       <c r="E21" t="n">
-        <v>6426.128757906712</v>
+        <v>6485.64123931475</v>
       </c>
       <c r="F21" t="n">
-        <v>-250.0916298891243</v>
+        <v>-272.9756650227428</v>
       </c>
     </row>
     <row r="22">
@@ -986,13 +986,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3894.6</v>
+        <v>543.8</v>
       </c>
       <c r="E22" t="n">
-        <v>4.0983</v>
+        <v>-496</v>
       </c>
       <c r="F22" t="n">
-        <v>-3890.5017</v>
+        <v>-1039.8</v>
       </c>
     </row>
     <row r="23">
@@ -1012,13 +1012,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9606.9</v>
+        <v>12351</v>
       </c>
       <c r="E23" t="n">
-        <v>9606.9</v>
+        <v>29949.7</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>17598.7</v>
       </c>
     </row>
     <row r="24">
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.950204222540247</v>
+        <v>1.043689938580875</v>
       </c>
       <c r="E24" t="n">
-        <v>1.066223381697571</v>
+        <v>0.6383011751611313</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.8839808408426764</v>
+        <v>-0.4053887634197438</v>
       </c>
     </row>
     <row r="25">
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>0.0011883541295306</v>
       </c>
       <c r="E25" t="n">
-        <v>0.03782707622298066</v>
+        <v>0.05923344947735192</v>
       </c>
       <c r="F25" t="n">
-        <v>0.03782707622298066</v>
+        <v>0.05804509534782132</v>
       </c>
     </row>
   </sheetData>
@@ -1116,13 +1116,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8681.620000000001</v>
+        <v>8165.059999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>8.681620000000001</v>
+        <v>8.16506</v>
       </c>
       <c r="D2" t="n">
-        <v>-8672.938380000001</v>
+        <v>-8156.894939999999</v>
       </c>
     </row>
     <row r="3">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8247.926666666666</v>
+        <v>8878.549999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>8.247926666666666</v>
+        <v>8.878550000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>-8239.678739999999</v>
+        <v>-8869.67145</v>
       </c>
     </row>
     <row r="4">
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8425.460000000001</v>
+        <v>8062.719999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>8.425459999999999</v>
+        <v>8.062720000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>-8417.034540000001</v>
+        <v>-8054.657279999999</v>
       </c>
     </row>
     <row r="5">
@@ -1164,13 +1164,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6933.455555555555</v>
+        <v>7376</v>
       </c>
       <c r="C5" t="n">
-        <v>6.933455555555556</v>
+        <v>7.376</v>
       </c>
       <c r="D5" t="n">
-        <v>-6926.5221</v>
+        <v>-7368.624</v>
       </c>
     </row>
     <row r="6">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6712.571428571428</v>
+        <v>6316.553846153846</v>
       </c>
       <c r="C6" t="n">
-        <v>6.712571428571429</v>
+        <v>6.316553846153846</v>
       </c>
       <c r="D6" t="n">
-        <v>-6705.858857142857</v>
+        <v>-6310.237292307693</v>
       </c>
     </row>
     <row r="7">
@@ -1196,13 +1196,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6546.590909090909</v>
+        <v>7065.954545454545</v>
       </c>
       <c r="C7" t="n">
-        <v>6.546590909090909</v>
+        <v>7.065954545454545</v>
       </c>
       <c r="D7" t="n">
-        <v>-6540.044318181818</v>
+        <v>-7058.88859090909</v>
       </c>
     </row>
     <row r="8">
@@ -1212,13 +1212,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8500.41</v>
+        <v>9138.33</v>
       </c>
       <c r="C8" t="n">
-        <v>8.500409999999999</v>
+        <v>9.13833</v>
       </c>
       <c r="D8" t="n">
-        <v>-8491.909589999999</v>
+        <v>-9129.19167</v>
       </c>
     </row>
     <row r="9">
@@ -1228,13 +1228,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7134.491666666666</v>
+        <v>7311.254545454546</v>
       </c>
       <c r="C9" t="n">
-        <v>7.134491666666666</v>
+        <v>7.311254545454545</v>
       </c>
       <c r="D9" t="n">
-        <v>-7127.357174999999</v>
+        <v>-7303.943290909092</v>
       </c>
     </row>
     <row r="10">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6655.588888888889</v>
+        <v>6749.666666666667</v>
       </c>
       <c r="C10" t="n">
-        <v>6.655588888888889</v>
+        <v>6.749666666666666</v>
       </c>
       <c r="D10" t="n">
-        <v>-6648.9333</v>
+        <v>-6742.917</v>
       </c>
     </row>
     <row r="11">
@@ -1260,13 +1260,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7717.127272727273</v>
+        <v>8286.263636363636</v>
       </c>
       <c r="C11" t="n">
-        <v>7.717127272727273</v>
+        <v>8.286263636363635</v>
       </c>
       <c r="D11" t="n">
-        <v>-7709.410145454545</v>
+        <v>-8277.977372727271</v>
       </c>
     </row>
     <row r="12">
@@ -1276,13 +1276,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7278.066666666667</v>
+        <v>6885.066666666667</v>
       </c>
       <c r="C12" t="n">
-        <v>7.278066666666667</v>
+        <v>6.885066666666667</v>
       </c>
       <c r="D12" t="n">
-        <v>-7270.7886</v>
+        <v>-6878.1816</v>
       </c>
     </row>
     <row r="13">
@@ -1292,13 +1292,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8621.976923076923</v>
+        <v>8145.746153846154</v>
       </c>
       <c r="C13" t="n">
-        <v>8.621976923076923</v>
+        <v>8.145746153846154</v>
       </c>
       <c r="D13" t="n">
-        <v>-8613.354946153846</v>
+        <v>-8137.600407692308</v>
       </c>
     </row>
     <row r="14">
@@ -1308,13 +1308,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8337.488888888889</v>
+        <v>7950.325</v>
       </c>
       <c r="C14" t="n">
-        <v>8.33748888888889</v>
+        <v>7.950325</v>
       </c>
       <c r="D14" t="n">
-        <v>-8329.151400000001</v>
+        <v>-7942.374675</v>
       </c>
     </row>
     <row r="15">
@@ -1324,13 +1324,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8545.253846153846</v>
+        <v>8731.830769230768</v>
       </c>
       <c r="C15" t="n">
-        <v>8.545253846153846</v>
+        <v>8.73183076923077</v>
       </c>
       <c r="D15" t="n">
-        <v>-8536.708592307692</v>
+        <v>-8723.098938461537</v>
       </c>
     </row>
     <row r="16">
@@ -1340,13 +1340,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6674.971428571429</v>
+        <v>6820.25</v>
       </c>
       <c r="C16" t="n">
-        <v>6.674971428571429</v>
+        <v>6.820250000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>-6668.296457142857</v>
+        <v>-6813.42975</v>
       </c>
     </row>
     <row r="17">
@@ -1356,13 +1356,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8187.166666666667</v>
+        <v>8269.586666666666</v>
       </c>
       <c r="C17" t="n">
-        <v>8.187166666666666</v>
+        <v>8.269586666666667</v>
       </c>
       <c r="D17" t="n">
-        <v>-8178.9795</v>
+        <v>-8261.317079999999</v>
       </c>
     </row>
     <row r="18">
@@ -1372,13 +1372,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7867.724999999999</v>
+        <v>8173.008333333334</v>
       </c>
       <c r="C18" t="n">
-        <v>7.867725</v>
+        <v>8.173008333333334</v>
       </c>
       <c r="D18" t="n">
-        <v>-7859.857274999999</v>
+        <v>-8164.835325000001</v>
       </c>
     </row>
     <row r="19">
@@ -1388,13 +1388,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6507.607142857143</v>
+        <v>6687.746153846154</v>
       </c>
       <c r="C19" t="n">
-        <v>6.507607142857142</v>
+        <v>6.687746153846154</v>
       </c>
       <c r="D19" t="n">
-        <v>-6501.099535714286</v>
+        <v>-6681.058407692308</v>
       </c>
     </row>
     <row r="20">
@@ -1404,13 +1404,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8814.74</v>
+        <v>8534.128571428571</v>
       </c>
       <c r="C20" t="n">
-        <v>8.81474</v>
+        <v>8.534128571428571</v>
       </c>
       <c r="D20" t="n">
-        <v>-8805.92526</v>
+        <v>-8525.594442857142</v>
       </c>
     </row>
     <row r="21">
@@ -1420,13 +1420,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>8645.98</v>
+        <v>8191.35</v>
       </c>
       <c r="C21" t="n">
-        <v>8.64598</v>
+        <v>8.19135</v>
       </c>
       <c r="D21" t="n">
-        <v>-8637.33402</v>
+        <v>-8183.15865</v>
       </c>
     </row>
     <row r="22">
@@ -1436,13 +1436,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8154.877777777777</v>
+        <v>8743.4</v>
       </c>
       <c r="C22" t="n">
-        <v>8.154877777777777</v>
+        <v>8.743399999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>-8146.722899999999</v>
+        <v>-8734.6566</v>
       </c>
     </row>
     <row r="23">
@@ -1452,13 +1452,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6729.280000000001</v>
+        <v>6084.33</v>
       </c>
       <c r="C23" t="n">
-        <v>6.72928</v>
+        <v>6.08433</v>
       </c>
       <c r="D23" t="n">
-        <v>-6722.550720000001</v>
+        <v>-6078.24567</v>
       </c>
     </row>
     <row r="24">
@@ -1468,13 +1468,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>7341.726666666666</v>
+        <v>6488.506666666667</v>
       </c>
       <c r="C24" t="n">
-        <v>7.341726666666667</v>
+        <v>6.488506666666667</v>
       </c>
       <c r="D24" t="n">
-        <v>-7334.38494</v>
+        <v>-6482.018160000001</v>
       </c>
     </row>
     <row r="25">
@@ -1484,13 +1484,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6829.02</v>
+        <v>7313.990000000001</v>
       </c>
       <c r="C25" t="n">
-        <v>6.82902</v>
+        <v>7.31399</v>
       </c>
       <c r="D25" t="n">
-        <v>-6822.190979999999</v>
+        <v>-7306.676010000001</v>
       </c>
     </row>
     <row r="26">
@@ -1500,13 +1500,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7382.971428571429</v>
+        <v>7206.338461538461</v>
       </c>
       <c r="C26" t="n">
-        <v>7.382971428571429</v>
+        <v>7.206338461538461</v>
       </c>
       <c r="D26" t="n">
-        <v>-7375.588457142858</v>
+        <v>-7199.132123076923</v>
       </c>
     </row>
     <row r="27">
@@ -1516,13 +1516,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9504.766666666666</v>
+        <v>8746.9375</v>
       </c>
       <c r="C27" t="n">
-        <v>9.504766666666667</v>
+        <v>8.746937500000001</v>
       </c>
       <c r="D27" t="n">
-        <v>-9495.2619</v>
+        <v>-8738.1905625</v>
       </c>
     </row>
     <row r="28">
@@ -1532,13 +1532,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>7894.809090909091</v>
+        <v>8262.581818181818</v>
       </c>
       <c r="C28" t="n">
-        <v>7.894809090909091</v>
+        <v>8.262581818181818</v>
       </c>
       <c r="D28" t="n">
-        <v>-7886.914281818182</v>
+        <v>-8254.319236363635</v>
       </c>
     </row>
     <row r="29">
@@ -1548,13 +1548,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6690.954545454545</v>
+        <v>6311.227272727273</v>
       </c>
       <c r="C29" t="n">
-        <v>6.690954545454545</v>
+        <v>6.311227272727273</v>
       </c>
       <c r="D29" t="n">
-        <v>-6684.26359090909</v>
+        <v>-6304.916045454545</v>
       </c>
     </row>
     <row r="30">
@@ -1564,13 +1564,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6962.13125</v>
+        <v>6776.51875</v>
       </c>
       <c r="C30" t="n">
-        <v>6.96213125</v>
+        <v>6.77651875</v>
       </c>
       <c r="D30" t="n">
-        <v>-6955.16911875</v>
+        <v>-6769.74223125</v>
       </c>
     </row>
     <row r="31">
@@ -1580,13 +1580,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7425.9</v>
+        <v>6555.177777777778</v>
       </c>
       <c r="C31" t="n">
-        <v>7.4259</v>
+        <v>6.555177777777778</v>
       </c>
       <c r="D31" t="n">
-        <v>-7418.474099999999</v>
+        <v>-6548.6226</v>
       </c>
     </row>
     <row r="32">
@@ -1596,13 +1596,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7867.627272727273</v>
+        <v>8094.836363636364</v>
       </c>
       <c r="C32" t="n">
-        <v>7.867627272727273</v>
+        <v>8.094836363636363</v>
       </c>
       <c r="D32" t="n">
-        <v>-7859.759645454546</v>
+        <v>-8086.741527272728</v>
       </c>
     </row>
     <row r="33">
@@ -1612,13 +1612,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>8181.176923076923</v>
+        <v>8754.353846153846</v>
       </c>
       <c r="C33" t="n">
-        <v>8.181176923076922</v>
+        <v>8.754353846153846</v>
       </c>
       <c r="D33" t="n">
-        <v>-8172.995746153846</v>
+        <v>-8745.599492307692</v>
       </c>
     </row>
     <row r="34">
@@ -1628,13 +1628,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>8002.233333333334</v>
+        <v>8265.557142857144</v>
       </c>
       <c r="C34" t="n">
-        <v>8.002233333333333</v>
+        <v>8.265557142857142</v>
       </c>
       <c r="D34" t="n">
-        <v>-7994.2311</v>
+        <v>-8257.291585714287</v>
       </c>
     </row>
     <row r="35">
@@ -1644,13 +1644,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>5932.215384615385</v>
+        <v>6939.238461538462</v>
       </c>
       <c r="C35" t="n">
-        <v>5.932215384615385</v>
+        <v>6.939238461538461</v>
       </c>
       <c r="D35" t="n">
-        <v>-5926.28316923077</v>
+        <v>-6932.299223076923</v>
       </c>
     </row>
     <row r="36">
@@ -1660,13 +1660,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>6360.972727272727</v>
+        <v>7354.409090909091</v>
       </c>
       <c r="C36" t="n">
-        <v>6.360972727272727</v>
+        <v>7.35440909090909</v>
       </c>
       <c r="D36" t="n">
-        <v>-6354.611754545454</v>
+        <v>-7347.054681818182</v>
       </c>
     </row>
     <row r="37">
@@ -1676,13 +1676,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>6513.193333333333</v>
+        <v>7016.278571428571</v>
       </c>
       <c r="C37" t="n">
-        <v>6.513193333333334</v>
+        <v>7.016278571428572</v>
       </c>
       <c r="D37" t="n">
-        <v>-6506.680139999999</v>
+        <v>-7009.262292857143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
P20: tanam jenis uji shear (generator v3, parser, spec, views, cek silang, Report); data push tidak berubah
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YpKXFN1b3yUWd7Emtd6MU
</commit_message>
<xml_diff>
--- a/project/outputs/reconciliation.xlsx
+++ b/project/outputs/reconciliation.xlsx
@@ -466,13 +466,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3401</v>
+        <v>3399</v>
       </c>
       <c r="E2" t="n">
         <v>3528</v>
       </c>
       <c r="F2" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8581.919288444575</v>
+        <v>8581.898205354517</v>
       </c>
       <c r="E3" t="n">
-        <v>8305.5497125</v>
+        <v>8305.255834948981</v>
       </c>
       <c r="F3" t="n">
-        <v>-276.3695759445745</v>
+        <v>-276.642370405536</v>
       </c>
     </row>
     <row r="4">
@@ -570,13 +570,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.734510112171457</v>
+        <v>2.733790999277372</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9022634204720315</v>
+        <v>0.9018957531049863</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.832246691699425</v>
+        <v>-1.831895246172386</v>
       </c>
     </row>
     <row r="7">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3721</v>
+        <v>3722</v>
       </c>
       <c r="E8" t="n">
         <v>3892</v>
       </c>
       <c r="F8" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9">
@@ -648,13 +648,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7151.974872346143</v>
+        <v>7151.913621708759</v>
       </c>
       <c r="E9" t="n">
         <v>7057.344121402878</v>
       </c>
       <c r="F9" t="n">
-        <v>-94.63075094326541</v>
+        <v>-94.56950030588087</v>
       </c>
     </row>
     <row r="10">
@@ -726,13 +726,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.123856983079873</v>
+        <v>2.124100557464248</v>
       </c>
       <c r="E12" t="n">
         <v>0.7704692736255384</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.353387709454334</v>
+        <v>-1.353631283838709</v>
       </c>
     </row>
     <row r="13">
@@ -807,10 +807,10 @@
         <v>8300.667233294256</v>
       </c>
       <c r="E15" t="n">
-        <v>8094.700690159352</v>
+        <v>8092.149669751188</v>
       </c>
       <c r="F15" t="n">
-        <v>-205.966543134904</v>
+        <v>-208.5175635430678</v>
       </c>
     </row>
     <row r="16">
@@ -885,10 +885,10 @@
         <v>2.564694707772915</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8038623471140007</v>
+        <v>0.8026100991589501</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.760832360658914</v>
+        <v>-1.762084608613965</v>
       </c>
     </row>
     <row r="19">
@@ -911,10 +911,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0.06094492591557171</v>
+        <v>0.06122448979591837</v>
       </c>
       <c r="F19" t="n">
-        <v>0.06094492591557171</v>
+        <v>0.06122448979591837</v>
       </c>
     </row>
     <row r="20">
@@ -934,13 +934,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3366</v>
+        <v>3359</v>
       </c>
       <c r="E20" t="n">
         <v>3444</v>
       </c>
       <c r="F20" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21">
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6758.616904337493</v>
+        <v>6758.595980946711</v>
       </c>
       <c r="E21" t="n">
         <v>6485.64123931475</v>
       </c>
       <c r="F21" t="n">
-        <v>-272.9756650227428</v>
+        <v>-272.954741631961</v>
       </c>
     </row>
     <row r="22">
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.043689938580875</v>
+        <v>1.043054192288527</v>
       </c>
       <c r="E24" t="n">
         <v>0.6383011751611313</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.4053887634197438</v>
+        <v>-0.4047530171273958</v>
       </c>
     </row>
     <row r="25">
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.0011883541295306</v>
+        <v>0.001190830604346532</v>
       </c>
       <c r="E25" t="n">
         <v>0.05923344947735192</v>
       </c>
       <c r="F25" t="n">
-        <v>0.05804509534782132</v>
+        <v>0.05804261887300538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>